<commit_message>
updated app logo + proifle page username ändern
</commit_message>
<xml_diff>
--- a/Dokumentation/Organisation/DS_Aufwandsschaetzung_1.0.xlsx
+++ b/Dokumentation/Organisation/DS_Aufwandsschaetzung_1.0.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Drive Sense\Dokumentation\Organisation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6DC6345-0457-4547-9FFF-79A24C9D58EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FF1AFD7-9DCB-4EC0-A81F-031DB741B8F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="16440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Aufwandsschätzung" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="0">Aufwandsschätzung!$A$1:$J$49</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">Aufwandsschätzung!$1:$1</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="130">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="102">
   <si>
     <t>Ist-Stunden</t>
   </si>
@@ -343,90 +343,6 @@
   </si>
   <si>
     <t>Aufgabenbezeichnung</t>
-  </si>
-  <si>
-    <t>5.1.1.3.1</t>
-  </si>
-  <si>
-    <t>Login-Formular (HTML/CSS) implementieren</t>
-  </si>
-  <si>
-    <t>5.1.1.3.2</t>
-  </si>
-  <si>
-    <t>Register-Formular implementieren</t>
-  </si>
-  <si>
-    <t>5.1.1.3.3</t>
-  </si>
-  <si>
-    <t>Session-/Token-Handling im Browser</t>
-  </si>
-  <si>
-    <t>5.1.1.3.4</t>
-  </si>
-  <si>
-    <t>Fehlerbehandlung &amp; Validierungsmeldungen</t>
-  </si>
-  <si>
-    <t>5.1.2.4.1</t>
-  </si>
-  <si>
-    <t>Login-Screen implementieren</t>
-  </si>
-  <si>
-    <t>5.1.2.4.2</t>
-  </si>
-  <si>
-    <t>Register-Screen implementieren</t>
-  </si>
-  <si>
-    <t>5.1.2.4.3</t>
-  </si>
-  <si>
-    <t>Sichere Token-Speicherung (SecureStorage)</t>
-  </si>
-  <si>
-    <t>5.1.2.4.4</t>
-  </si>
-  <si>
-    <t>Auto-Login / Session-Persistenz</t>
-  </si>
-  <si>
-    <t>5.1.2.4.5</t>
-  </si>
-  <si>
-    <t>Fehlerbehandlung &amp; UX-Feedback</t>
-  </si>
-  <si>
-    <t>5.2.2.1</t>
-  </si>
-  <si>
-    <t>REST-API Endpunkte definieren &amp; dokumentieren</t>
-  </si>
-  <si>
-    <t>5.2.2.2</t>
-  </si>
-  <si>
-    <t>API-Endpunkte für die Web-App implementieren</t>
-  </si>
-  <si>
-    <t>5.2.2.3</t>
-  </si>
-  <si>
-    <t>API-Endpunkte für die App implementieren</t>
-  </si>
-  <si>
-    <t>5.2.2.4</t>
-  </si>
-  <si>
-    <t>JWT / Authentifizierung serverseitig implementieren</t>
-  </si>
-  <si>
-    <t>5.2.2.5</t>
-  </si>
-  <si>
-    <t>API-Tests schreiben</t>
   </si>
 </sst>
 </file>
@@ -442,26 +358,25 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="18"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="4">
@@ -474,13 +389,13 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF0070C0"/>
-        <bgColor rgb="FF008080"/>
+        <bgColor rgb="FFFFD966"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.39988402966399123"/>
-        <bgColor rgb="FF9999FF"/>
+        <fgColor theme="4" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -515,27 +430,59 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Prozent" xfId="1" builtinId="5"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="3">
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="0" formatCode="General"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFD966"/>
+          <bgColor rgb="FF0070C0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -549,19 +496,25 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8DD183D6-DB0F-449B-89C5-C88BDFF020C3}" name="Tabelle22" displayName="Tabelle22" ref="A1:J62" totalsRowShown="0">
-  <autoFilter ref="A1:J62" xr:uid="{8DD183D6-DB0F-449B-89C5-C88BDFF020C3}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1449D87B-F32E-4C26-BAE3-4976F948F37B}" name="Tabelle2" displayName="Tabelle2" ref="A1:J48" totalsRowShown="0" headerRowDxfId="2">
+  <autoFilter ref="A1:J48" xr:uid="{1449D87B-F32E-4C26-BAE3-4976F948F37B}"/>
   <tableColumns count="10">
-    <tableColumn id="1" xr3:uid="{8E9E6F6C-782A-4F8C-8799-944A24E47CDA}" name="Nr."/>
-    <tableColumn id="2" xr3:uid="{475A8BCA-BB53-4CB0-B874-246311335731}" name="Aufgabenbezeichnung"/>
-    <tableColumn id="3" xr3:uid="{70420603-B613-4C29-8797-85C845698842}" name="Eric"/>
-    <tableColumn id="4" xr3:uid="{DDB561E8-4D15-4123-B1A0-400281A69B16}" name="Christof"/>
-    <tableColumn id="5" xr3:uid="{9118E39F-5251-4FFF-AA33-D4B6252CF687}" name="Daniel"/>
-    <tableColumn id="6" xr3:uid="{75D1BFFF-944E-493C-9F03-363D6A56E467}" name="Niklas"/>
-    <tableColumn id="7" xr3:uid="{054DCE2D-EF46-4CCA-A024-A88E9CC372B2}" name="Ø Schätzung (Soll-MA-Stunden)"/>
-    <tableColumn id="8" xr3:uid="{D930034A-04D4-4C9A-B07C-74C6ED92701E}" name="Ist-Stunden"/>
-    <tableColumn id="9" xr3:uid="{8522511C-8106-463A-92C8-DE128350C1FB}" name="Abweichung (Std.)"/>
-    <tableColumn id="10" xr3:uid="{3C4DAF9C-B97B-4874-83CC-4CA3B6D45A9F}" name="Abweichung (%)"/>
+    <tableColumn id="1" xr3:uid="{E8F675F9-1C93-40E7-8E9E-8B166EAF1C74}" name="Nr."/>
+    <tableColumn id="2" xr3:uid="{B6EE27EE-76B8-465C-8058-B5C39BDC2371}" name="Aufgabenbezeichnung"/>
+    <tableColumn id="3" xr3:uid="{1890D48C-756E-4C90-B565-6D8A9FF058EC}" name="Eric"/>
+    <tableColumn id="4" xr3:uid="{DCBC915B-FBA7-408B-965C-F00644F48D7D}" name="Christof"/>
+    <tableColumn id="5" xr3:uid="{DCC1A44A-6BBE-493F-851A-578DCF9BE266}" name="Daniel"/>
+    <tableColumn id="6" xr3:uid="{FC590683-3EA5-4EC9-B287-5336B779348D}" name="Niklas"/>
+    <tableColumn id="7" xr3:uid="{15D9E014-198F-4E07-BF5C-FDDFE788A919}" name="Ø Schätzung (Soll-MA-Stunden)">
+      <calculatedColumnFormula>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="8" xr3:uid="{A739C55C-971E-4CD4-B52C-0D40350E395B}" name="Ist-Stunden"/>
+    <tableColumn id="9" xr3:uid="{0895D37D-EA7F-47C8-AD16-6143B28C06CC}" name="Abweichung (Std.)" dataDxfId="1">
+      <calculatedColumnFormula>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</calculatedColumnFormula>
+    </tableColumn>
+    <tableColumn id="10" xr3:uid="{64A9A77C-10FA-460A-B67E-CD87C00870E6}" name="Abweichung (%)" dataDxfId="0">
+      <calculatedColumnFormula>Tabelle2[[#This Row],[Abweichung (Std.)]]</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -855,7 +808,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J64"/>
+  <dimension ref="A1:J50"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
@@ -869,34 +822,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="1" t="s">
         <v>100</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="1" t="s">
         <v>101</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="E1" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="1" t="s">
         <v>75</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="I1" s="3" t="s">
+      <c r="I1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
@@ -924,15 +877,15 @@
         <v>30</v>
       </c>
       <c r="G2">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>33.5</v>
       </c>
       <c r="I2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-33.5</v>
       </c>
       <c r="J2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-33.5</v>
       </c>
     </row>
@@ -956,18 +909,18 @@
         <v>2.5</v>
       </c>
       <c r="G3">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>2.5</v>
       </c>
       <c r="H3">
         <v>0.79</v>
       </c>
       <c r="I3">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-1.71</v>
       </c>
-      <c r="J3" s="4">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+      <c r="J3" s="7">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-1.71</v>
       </c>
     </row>
@@ -991,20 +944,20 @@
         <v>4</v>
       </c>
       <c r="G4">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>6.25</v>
       </c>
       <c r="I4">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-6.25</v>
       </c>
       <c r="J4">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-6.25</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B5" t="s">
@@ -1023,23 +976,23 @@
         <v>6</v>
       </c>
       <c r="G5">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>6.5</v>
       </c>
       <c r="H5">
         <v>4.76</v>
       </c>
       <c r="I5">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-1.7400000000000002</v>
       </c>
       <c r="J5">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-1.7400000000000002</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B6" t="s">
@@ -1058,20 +1011,20 @@
         <v>2.5</v>
       </c>
       <c r="G6">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>2</v>
       </c>
       <c r="I6">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-2</v>
       </c>
       <c r="J6">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-2</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>76</v>
       </c>
       <c r="B7" t="s">
@@ -1090,23 +1043,23 @@
         <v>6</v>
       </c>
       <c r="G7">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>6.5</v>
       </c>
       <c r="H7">
         <v>3.56</v>
       </c>
       <c r="I7">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-2.94</v>
       </c>
       <c r="J7">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-2.94</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>92</v>
       </c>
       <c r="B8" t="s">
@@ -1125,52 +1078,52 @@
         <v>9</v>
       </c>
       <c r="G8">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>9.75</v>
       </c>
       <c r="I8">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-9.75</v>
       </c>
       <c r="J8">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-9.75</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="A9" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C9" s="2">
-        <f>SUM(C10:C14)</f>
+      <c r="C9" s="3">
+        <f t="shared" ref="C9:F9" si="0">SUM(C10:C14)</f>
         <v>61</v>
       </c>
-      <c r="D9" s="2">
-        <f>SUM(D10:D14)</f>
+      <c r="D9" s="3">
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="E9" s="2">
-        <f>SUM(E10:E14)</f>
+      <c r="E9" s="3">
+        <f t="shared" si="0"/>
         <v>64</v>
       </c>
-      <c r="F9" s="2">
-        <f>SUM(F10:F14)</f>
+      <c r="F9" s="3">
+        <f t="shared" si="0"/>
         <v>59</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="3">
         <f>SUM(G10:G14)</f>
         <v>60.75</v>
       </c>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-60.75</v>
       </c>
-      <c r="J9" s="2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+      <c r="J9" s="3">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-60.75</v>
       </c>
     </row>
@@ -1194,18 +1147,18 @@
         <v>15</v>
       </c>
       <c r="G10">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>14.25</v>
       </c>
       <c r="H10">
         <v>11.5</v>
       </c>
       <c r="I10">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-2.75</v>
       </c>
       <c r="J10">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-2.75</v>
       </c>
     </row>
@@ -1229,18 +1182,18 @@
         <v>7</v>
       </c>
       <c r="G11">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>6.5</v>
       </c>
       <c r="H11">
         <v>9.5</v>
       </c>
       <c r="I11">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>3</v>
       </c>
       <c r="J11">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>3</v>
       </c>
     </row>
@@ -1264,23 +1217,23 @@
         <v>16</v>
       </c>
       <c r="G12">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>14.25</v>
       </c>
       <c r="H12">
         <v>10</v>
       </c>
       <c r="I12">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-4.25</v>
       </c>
       <c r="J12">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-4.25</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A13" s="1" t="s">
+      <c r="A13" s="2" t="s">
         <v>94</v>
       </c>
       <c r="B13" t="s">
@@ -1299,20 +1252,20 @@
         <v>18</v>
       </c>
       <c r="G13">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>21.25</v>
       </c>
       <c r="I13">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-21.25</v>
       </c>
       <c r="J13">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-21.25</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A14" s="1" t="s">
+      <c r="A14" s="2" t="s">
         <v>98</v>
       </c>
       <c r="B14" t="s">
@@ -1331,55 +1284,55 @@
         <v>3</v>
       </c>
       <c r="G14">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>4.5</v>
       </c>
       <c r="H14">
         <v>8.59</v>
       </c>
       <c r="I14">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>4.09</v>
       </c>
       <c r="J14">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>4.09</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A15" s="2" t="s">
+      <c r="A15" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C15" s="2">
+      <c r="C15" s="3">
         <f>SUM(C16:C18)</f>
         <v>10</v>
       </c>
-      <c r="D15" s="2">
-        <f>SUM(D16:D18)</f>
+      <c r="D15" s="3">
+        <f t="shared" ref="D15:G15" si="1">SUM(D16:D18)</f>
         <v>10</v>
       </c>
-      <c r="E15" s="2">
-        <f>SUM(E16:E18)</f>
+      <c r="E15" s="3">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="F15" s="2">
-        <f>SUM(F16:F18)</f>
+      <c r="F15" s="3">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="G15" s="2">
-        <f>SUM(G16:G18)</f>
+      <c r="G15" s="3">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="H15" s="2"/>
-      <c r="I15" s="2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-10</v>
       </c>
-      <c r="J15" s="2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+      <c r="J15" s="3">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-10</v>
       </c>
     </row>
@@ -1403,15 +1356,15 @@
         <v>3</v>
       </c>
       <c r="G16">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>2.75</v>
       </c>
       <c r="I16">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-2.75</v>
       </c>
       <c r="J16">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-2.75</v>
       </c>
     </row>
@@ -1435,15 +1388,15 @@
         <v>3</v>
       </c>
       <c r="G17">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>2.75</v>
       </c>
       <c r="I17">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-2.75</v>
       </c>
       <c r="J17">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-2.75</v>
       </c>
     </row>
@@ -1467,52 +1420,52 @@
         <v>4</v>
       </c>
       <c r="G18">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>4.5</v>
       </c>
       <c r="I18">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-4.5</v>
       </c>
       <c r="J18">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-4.5</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A19" s="2" t="s">
+      <c r="A19" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="C19" s="2">
+      <c r="C19" s="3">
         <f>SUM(C20:C24)</f>
         <v>19</v>
       </c>
-      <c r="D19" s="2">
-        <f>SUM(D20:D24)</f>
+      <c r="D19" s="3">
+        <f t="shared" ref="D19:G19" si="2">SUM(D20:D24)</f>
         <v>20.5</v>
       </c>
-      <c r="E19" s="2">
-        <f>SUM(E20:E24)</f>
+      <c r="E19" s="3">
+        <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="F19" s="2">
-        <f>SUM(F20:F24)</f>
+      <c r="F19" s="3">
+        <f t="shared" si="2"/>
         <v>17.5</v>
       </c>
-      <c r="G19" s="2">
-        <f>SUM(G20:G24)</f>
+      <c r="G19" s="3">
+        <f t="shared" si="2"/>
         <v>18.25</v>
       </c>
-      <c r="H19" s="2"/>
-      <c r="I19" s="2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-18.25</v>
       </c>
-      <c r="J19" s="2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+      <c r="J19" s="3">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-18.25</v>
       </c>
     </row>
@@ -1536,18 +1489,18 @@
         <v>1</v>
       </c>
       <c r="G20">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>1.5</v>
       </c>
       <c r="H20">
         <v>1.56</v>
       </c>
       <c r="I20">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>6.0000000000000053E-2</v>
       </c>
       <c r="J20">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>6.0000000000000053E-2</v>
       </c>
     </row>
@@ -1571,15 +1524,15 @@
         <v>0.5</v>
       </c>
       <c r="G21">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>0.75</v>
       </c>
       <c r="I21">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-0.75</v>
       </c>
       <c r="J21">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-0.75</v>
       </c>
     </row>
@@ -1603,15 +1556,15 @@
         <v>6</v>
       </c>
       <c r="G22">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>6.5</v>
       </c>
       <c r="I22">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-6.5</v>
       </c>
       <c r="J22">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-6.5</v>
       </c>
     </row>
@@ -1635,15 +1588,15 @@
         <v>4</v>
       </c>
       <c r="G23">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>3.5</v>
       </c>
       <c r="I23">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-3.5</v>
       </c>
       <c r="J23">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-3.5</v>
       </c>
     </row>
@@ -1667,52 +1620,52 @@
         <v>6</v>
       </c>
       <c r="G24">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>6</v>
       </c>
       <c r="I24">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-6</v>
       </c>
       <c r="J24">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-6</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A25" s="2" t="s">
+      <c r="A25" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C25" s="2">
-        <f>C26+C45</f>
+      <c r="C25" s="3">
+        <f>C26+C36</f>
         <v>209</v>
       </c>
-      <c r="D25" s="2">
-        <f>D26+D45</f>
+      <c r="D25" s="3">
+        <f t="shared" ref="D25:F25" si="3">D26+D36</f>
         <v>272</v>
       </c>
-      <c r="E25" s="2">
-        <f>E26+E45</f>
+      <c r="E25" s="3">
+        <f t="shared" si="3"/>
         <v>201</v>
       </c>
-      <c r="F25" s="2">
-        <f>F26+F45</f>
+      <c r="F25" s="3">
+        <f t="shared" si="3"/>
         <v>254</v>
       </c>
-      <c r="G25" s="2">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+      <c r="G25" s="3">
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>234</v>
       </c>
-      <c r="H25" s="2"/>
-      <c r="I25" s="2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-234</v>
       </c>
-      <c r="J25" s="2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+      <c r="J25" s="3">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-234</v>
       </c>
     </row>
@@ -1724,31 +1677,31 @@
         <v>83</v>
       </c>
       <c r="C26">
-        <f>C27+C35</f>
+        <f>C27+C31</f>
         <v>190</v>
       </c>
       <c r="D26">
-        <f>D27+D35</f>
+        <f>D27+D31</f>
         <v>250</v>
       </c>
       <c r="E26">
-        <f>E27+E35</f>
+        <f t="shared" ref="E26:F26" si="4">E27+E31</f>
         <v>178</v>
       </c>
       <c r="F26">
-        <f>F27+F35</f>
+        <f t="shared" si="4"/>
         <v>228</v>
       </c>
       <c r="G26">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>211.5</v>
       </c>
       <c r="I26">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-211.5</v>
       </c>
       <c r="J26">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-211.5</v>
       </c>
     </row>
@@ -1764,27 +1717,27 @@
         <v>55</v>
       </c>
       <c r="D27">
-        <f>SUM(D28:D30)</f>
+        <f t="shared" ref="D27:F27" si="5">SUM(D28:D30)</f>
         <v>66</v>
       </c>
       <c r="E27">
-        <f>SUM(E28:E30)</f>
+        <f t="shared" si="5"/>
         <v>48</v>
       </c>
       <c r="F27">
-        <f>SUM(F28:F30)</f>
+        <f t="shared" si="5"/>
         <v>66</v>
       </c>
       <c r="G27">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>58.75</v>
       </c>
       <c r="I27">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-58.75</v>
       </c>
       <c r="J27">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-58.75</v>
       </c>
     </row>
@@ -1808,15 +1761,15 @@
         <v>40</v>
       </c>
       <c r="G28">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>36.25</v>
       </c>
       <c r="I28">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-36.25</v>
       </c>
       <c r="J28">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-36.25</v>
       </c>
     </row>
@@ -1840,15 +1793,15 @@
         <v>20</v>
       </c>
       <c r="G29">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>17.75</v>
       </c>
       <c r="I29">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-17.75</v>
       </c>
       <c r="J29">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-17.75</v>
       </c>
     </row>
@@ -1860,1114 +1813,654 @@
         <v>50</v>
       </c>
       <c r="C30">
-        <f>SUM(C31:C34)</f>
         <v>5</v>
       </c>
       <c r="D30">
-        <f>SUM(D31:D34)</f>
         <v>5</v>
       </c>
       <c r="E30">
-        <f>SUM(E31:E34)</f>
         <v>3</v>
       </c>
       <c r="F30">
-        <f>SUM(F31:F34)</f>
         <v>6</v>
       </c>
       <c r="G30">
-        <f>AVERAGE(C30:F30)</f>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
         <v>4.75</v>
       </c>
       <c r="I30">
-        <f>H30-G30</f>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
         <v>-4.75</v>
       </c>
       <c r="J30">
-        <f>I30</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-4.75</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>102</v>
+        <v>51</v>
       </c>
       <c r="B31" t="s">
-        <v>103</v>
+        <v>52</v>
       </c>
       <c r="C31">
-        <v>1.5</v>
+        <f>SUM(C32:C35)</f>
+        <v>135</v>
       </c>
       <c r="D31">
-        <v>1.5</v>
+        <f t="shared" ref="D31:F31" si="6">SUM(D32:D35)</f>
+        <v>184</v>
       </c>
       <c r="E31">
-        <v>1</v>
+        <f t="shared" si="6"/>
+        <v>130</v>
       </c>
       <c r="F31">
-        <v>1.5</v>
+        <f t="shared" si="6"/>
+        <v>162</v>
       </c>
       <c r="G31">
-        <f>AVERAGE(C31:F31)</f>
-        <v>1.375</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>152.75</v>
       </c>
       <c r="I31">
-        <f>H31-G31</f>
-        <v>-1.375</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-152.75</v>
       </c>
       <c r="J31">
-        <f>I31</f>
-        <v>-1.375</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-152.75</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>104</v>
+        <v>53</v>
       </c>
       <c r="B32" t="s">
-        <v>105</v>
+        <v>46</v>
       </c>
       <c r="C32">
-        <v>1.5</v>
+        <v>45</v>
       </c>
       <c r="D32">
-        <v>1.5</v>
+        <v>60</v>
       </c>
       <c r="E32">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="F32">
-        <v>2</v>
+        <v>60</v>
       </c>
       <c r="G32">
-        <f>AVERAGE(C32:F32)</f>
-        <v>1.5</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>52.5</v>
       </c>
       <c r="I32">
-        <f>H32-G32</f>
-        <v>-1.5</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-52.5</v>
       </c>
       <c r="J32">
-        <f>I32</f>
-        <v>-1.5</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-52.5</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>106</v>
+        <v>54</v>
       </c>
       <c r="B33" t="s">
-        <v>107</v>
+        <v>48</v>
       </c>
       <c r="C33">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="D33">
-        <v>1</v>
+        <v>30</v>
       </c>
       <c r="E33">
-        <v>0.5</v>
+        <v>15</v>
       </c>
       <c r="F33">
-        <v>1.5</v>
+        <v>25</v>
       </c>
       <c r="G33">
-        <f>AVERAGE(C33:F33)</f>
-        <v>1</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>20.5</v>
       </c>
       <c r="I33">
-        <f>H33-G33</f>
-        <v>-1</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-20.5</v>
       </c>
       <c r="J33">
-        <f>I33</f>
-        <v>-1</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-20.5</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>108</v>
+        <v>55</v>
       </c>
       <c r="B34" t="s">
-        <v>109</v>
+        <v>56</v>
       </c>
       <c r="C34">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="D34">
-        <v>1</v>
+        <v>90</v>
       </c>
       <c r="E34">
-        <v>0.5</v>
+        <v>67</v>
       </c>
       <c r="F34">
-        <v>1</v>
+        <v>75</v>
       </c>
       <c r="G34">
-        <f>AVERAGE(C34:F34)</f>
-        <v>0.875</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>76.75</v>
       </c>
       <c r="I34">
-        <f>H34-G34</f>
-        <v>-0.875</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-76.75</v>
       </c>
       <c r="J34">
-        <f>I34</f>
-        <v>-0.875</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-76.75</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>51</v>
+        <v>78</v>
       </c>
       <c r="B35" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C35">
-        <f>SUM(C36:C39)</f>
-        <v>135</v>
+        <v>3</v>
       </c>
       <c r="D35">
-        <f>SUM(D36:D39)</f>
-        <v>184</v>
+        <v>4</v>
       </c>
       <c r="E35">
-        <f>SUM(E36:E39)</f>
-        <v>130</v>
+        <v>3</v>
       </c>
       <c r="F35">
-        <f>SUM(F36:F39)</f>
-        <v>162</v>
+        <v>2</v>
       </c>
       <c r="G35">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>152.75</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>3</v>
       </c>
       <c r="I35">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-152.75</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-3</v>
       </c>
       <c r="J35">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-152.75</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-3</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B36" t="s">
-        <v>46</v>
+        <v>84</v>
       </c>
       <c r="C36">
-        <v>45</v>
+        <f>SUM(C37:C39)</f>
+        <v>19</v>
       </c>
       <c r="D36">
-        <v>60</v>
+        <f t="shared" ref="D36:F36" si="7">SUM(D37:D39)</f>
+        <v>22</v>
       </c>
       <c r="E36">
-        <v>45</v>
+        <f t="shared" si="7"/>
+        <v>23</v>
       </c>
       <c r="F36">
-        <v>60</v>
+        <f t="shared" si="7"/>
+        <v>26</v>
       </c>
       <c r="G36">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>52.5</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>22.5</v>
       </c>
       <c r="I36">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-52.5</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-22.5</v>
       </c>
       <c r="J36">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-52.5</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-22.5</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B37" t="s">
-        <v>48</v>
+        <v>88</v>
       </c>
       <c r="C37">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D37">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="E37">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="F37">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="G37">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>20.5</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>6.75</v>
       </c>
       <c r="I37">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-20.5</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-6.75</v>
       </c>
       <c r="J37">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-20.5</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-6.75</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B38" t="s">
-        <v>56</v>
+        <v>89</v>
       </c>
       <c r="C38">
-        <v>75</v>
+        <v>7</v>
       </c>
       <c r="D38">
+        <v>8</v>
+      </c>
+      <c r="E38">
+        <v>9</v>
+      </c>
+      <c r="F38">
+        <v>9</v>
+      </c>
+      <c r="G38">
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>8.25</v>
+      </c>
+      <c r="I38">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-8.25</v>
+      </c>
+      <c r="J38">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-8.25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A39" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B39" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E38">
-        <v>67</v>
-      </c>
-      <c r="F38">
-        <v>75</v>
-      </c>
-      <c r="G38">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>76.75</v>
-      </c>
-      <c r="I38">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-76.75</v>
-      </c>
-      <c r="J38">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-76.75</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>78</v>
-      </c>
-      <c r="B39" t="s">
-        <v>50</v>
-      </c>
       <c r="C39">
-        <f>SUM(C40:C44)</f>
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="D39">
-        <f>SUM(D40:D44)</f>
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E39">
-        <f>SUM(E40:E44)</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F39">
-        <f>SUM(F40:F44)</f>
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="G39">
-        <f t="shared" ref="G39:G44" si="0">AVERAGE(C39:F39)</f>
-        <v>3</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>7.5</v>
       </c>
       <c r="I39">
-        <f t="shared" ref="I39:I44" si="1">H39-G39</f>
-        <v>-3</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-7.5</v>
       </c>
       <c r="J39">
-        <f t="shared" ref="J39:J44" si="2">I39</f>
-        <v>-3</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-7.5</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>110</v>
-      </c>
-      <c r="B40" t="s">
-        <v>111</v>
-      </c>
-      <c r="C40">
-        <v>0.75</v>
-      </c>
-      <c r="D40">
-        <v>1</v>
-      </c>
-      <c r="E40">
-        <v>0.75</v>
-      </c>
-      <c r="F40">
-        <v>0.5</v>
-      </c>
-      <c r="G40">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
-      </c>
-      <c r="I40">
-        <f t="shared" si="1"/>
-        <v>-0.75</v>
-      </c>
-      <c r="J40">
-        <f t="shared" si="2"/>
-        <v>-0.75</v>
+      <c r="A40" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B40" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C40" s="3">
+        <f>SUM(C41:C45)</f>
+        <v>47</v>
+      </c>
+      <c r="D40" s="3">
+        <f t="shared" ref="D40:G40" si="8">SUM(D41:D45)</f>
+        <v>43</v>
+      </c>
+      <c r="E40" s="3">
+        <f t="shared" si="8"/>
+        <v>44.5</v>
+      </c>
+      <c r="F40" s="3">
+        <f t="shared" si="8"/>
+        <v>33.5</v>
+      </c>
+      <c r="G40" s="3">
+        <f t="shared" si="8"/>
+        <v>42</v>
+      </c>
+      <c r="H40" s="3"/>
+      <c r="I40" s="3">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-42</v>
+      </c>
+      <c r="J40" s="3">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-42</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>112</v>
+        <v>62</v>
       </c>
       <c r="B41" t="s">
-        <v>113</v>
+        <v>87</v>
       </c>
       <c r="C41">
-        <v>0.75</v>
+        <v>4</v>
       </c>
       <c r="D41">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E41">
-        <v>0.75</v>
+        <v>7</v>
       </c>
       <c r="F41">
-        <v>0.5</v>
+        <v>5.5</v>
       </c>
       <c r="G41">
-        <f t="shared" si="0"/>
-        <v>0.75</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>5.125</v>
       </c>
       <c r="I41">
-        <f t="shared" si="1"/>
-        <v>-0.75</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-5.125</v>
       </c>
       <c r="J41">
-        <f t="shared" si="2"/>
-        <v>-0.75</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-5.125</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>114</v>
+        <v>63</v>
       </c>
       <c r="B42" t="s">
-        <v>115</v>
+        <v>86</v>
       </c>
       <c r="C42">
-        <v>0.5</v>
+        <v>6</v>
       </c>
       <c r="D42">
-        <v>0.75</v>
+        <v>8</v>
       </c>
       <c r="E42">
-        <v>0.5</v>
+        <v>6.5</v>
       </c>
       <c r="F42">
-        <v>0.5</v>
+        <v>5</v>
       </c>
       <c r="G42">
-        <f t="shared" si="0"/>
-        <v>0.5625</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>6.375</v>
       </c>
       <c r="I42">
-        <f t="shared" si="1"/>
-        <v>-0.5625</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-6.375</v>
       </c>
       <c r="J42">
-        <f t="shared" si="2"/>
-        <v>-0.5625</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-6.375</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>116</v>
+        <v>64</v>
       </c>
       <c r="B43" t="s">
-        <v>117</v>
+        <v>85</v>
       </c>
       <c r="C43">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="D43">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="E43">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="F43">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="G43">
-        <f t="shared" si="0"/>
-        <v>0.5</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>1.25</v>
       </c>
       <c r="I43">
-        <f t="shared" si="1"/>
-        <v>-0.5</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-1.25</v>
       </c>
       <c r="J43">
-        <f t="shared" si="2"/>
-        <v>-0.5</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-1.25</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>118</v>
+        <v>65</v>
       </c>
       <c r="B44" t="s">
-        <v>119</v>
+        <v>91</v>
       </c>
       <c r="C44">
-        <v>0.5</v>
+        <v>25</v>
       </c>
       <c r="D44">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="E44">
-        <v>0.5</v>
+        <v>20</v>
       </c>
       <c r="F44">
-        <v>0.25</v>
+        <v>15</v>
       </c>
       <c r="G44">
-        <f t="shared" si="0"/>
-        <v>0.4375</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>20</v>
       </c>
       <c r="I44">
-        <f t="shared" si="1"/>
-        <v>-0.4375</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-20</v>
       </c>
       <c r="J44">
-        <f t="shared" si="2"/>
-        <v>-0.4375</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-20</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>57</v>
+        <v>81</v>
       </c>
       <c r="B45" t="s">
-        <v>84</v>
+        <v>80</v>
       </c>
       <c r="C45">
-        <f>C46+C47+C53</f>
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="D45">
-        <f>D46+D47+D53</f>
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E45">
-        <f>E46+E47+E53</f>
-        <v>23</v>
+        <v>10</v>
       </c>
       <c r="F45">
-        <f>F46+F47+F53</f>
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="G45">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>22.5</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>9.25</v>
       </c>
       <c r="I45">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-22.5</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-9.25</v>
       </c>
       <c r="J45">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-22.5</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-9.25</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>58</v>
-      </c>
-      <c r="B46" t="s">
-        <v>88</v>
-      </c>
-      <c r="C46">
-        <v>6</v>
-      </c>
-      <c r="D46">
-        <v>6</v>
-      </c>
-      <c r="E46">
-        <v>7</v>
-      </c>
-      <c r="F46">
-        <v>8</v>
-      </c>
-      <c r="G46">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>6.75</v>
-      </c>
-      <c r="I46">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-6.75</v>
-      </c>
-      <c r="J46">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-6.75</v>
+      <c r="A46" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B46" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="C46" s="3">
+        <f>SUM(C47:C48)</f>
+        <v>36</v>
+      </c>
+      <c r="D46" s="3">
+        <f t="shared" ref="D46:G46" si="9">SUM(D47:D48)</f>
+        <v>28</v>
+      </c>
+      <c r="E46" s="3">
+        <f t="shared" si="9"/>
+        <v>32</v>
+      </c>
+      <c r="F46" s="3">
+        <f t="shared" si="9"/>
+        <v>25</v>
+      </c>
+      <c r="G46" s="3">
+        <f t="shared" si="9"/>
+        <v>30.25</v>
+      </c>
+      <c r="H46" s="3"/>
+      <c r="I46" s="3">
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-30.25</v>
+      </c>
+      <c r="J46" s="3">
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-30.25</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>59</v>
+        <v>68</v>
       </c>
       <c r="B47" t="s">
-        <v>89</v>
+        <v>69</v>
       </c>
       <c r="C47">
-        <f>SUM(C48:C52)</f>
-        <v>7</v>
+        <v>27</v>
       </c>
       <c r="D47">
-        <f>SUM(D48:D52)</f>
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E47">
-        <f>SUM(E48:E52)</f>
-        <v>9</v>
+        <v>22</v>
       </c>
       <c r="F47">
-        <f>SUM(F48:F52)</f>
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="G47">
-        <f t="shared" ref="G47:G52" si="3">AVERAGE(C47:F47)</f>
-        <v>8.25</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>21.5</v>
       </c>
       <c r="I47">
-        <f t="shared" ref="I47:I52" si="4">H47-G47</f>
-        <v>-8.25</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-21.5</v>
       </c>
       <c r="J47">
-        <f t="shared" ref="J47:J52" si="5">I47</f>
-        <v>-8.25</v>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
+        <v>-21.5</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>120</v>
+        <v>70</v>
       </c>
       <c r="B48" t="s">
-        <v>121</v>
+        <v>71</v>
       </c>
       <c r="C48">
-        <v>1.5</v>
+        <v>9</v>
       </c>
       <c r="D48">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="E48">
-        <v>1.5</v>
+        <v>10</v>
       </c>
       <c r="F48">
-        <v>1.5</v>
+        <v>8</v>
       </c>
       <c r="G48">
-        <f t="shared" si="3"/>
-        <v>1.5</v>
+        <f>AVERAGE(Tabelle2[[#This Row],[Niklas]]:Tabelle2[[#This Row],[Eric]])</f>
+        <v>8.75</v>
       </c>
       <c r="I48">
-        <f t="shared" si="4"/>
-        <v>-1.5</v>
+        <f>Tabelle2[[#This Row],[Ist-Stunden]]-Tabelle2[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <v>-8.75</v>
       </c>
       <c r="J48">
-        <f t="shared" si="5"/>
-        <v>-1.5</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>122</v>
-      </c>
-      <c r="B49" t="s">
-        <v>123</v>
-      </c>
-      <c r="C49">
-        <v>1.5</v>
-      </c>
-      <c r="D49">
-        <v>2</v>
-      </c>
-      <c r="E49">
-        <v>2</v>
-      </c>
-      <c r="F49">
-        <v>2</v>
-      </c>
-      <c r="G49">
-        <f t="shared" si="3"/>
-        <v>1.875</v>
-      </c>
-      <c r="I49">
-        <f t="shared" si="4"/>
-        <v>-1.875</v>
-      </c>
-      <c r="J49">
-        <f t="shared" si="5"/>
-        <v>-1.875</v>
-      </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>124</v>
-      </c>
-      <c r="B50" t="s">
-        <v>125</v>
-      </c>
-      <c r="C50">
-        <v>1.5</v>
-      </c>
-      <c r="D50">
-        <v>2</v>
-      </c>
-      <c r="E50">
-        <v>2.5</v>
-      </c>
-      <c r="F50">
-        <v>2.5</v>
-      </c>
-      <c r="G50">
-        <f t="shared" si="3"/>
-        <v>2.125</v>
-      </c>
-      <c r="I50">
-        <f t="shared" si="4"/>
-        <v>-2.125</v>
-      </c>
-      <c r="J50">
-        <f t="shared" si="5"/>
-        <v>-2.125</v>
-      </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>126</v>
-      </c>
-      <c r="B51" t="s">
-        <v>127</v>
-      </c>
-      <c r="C51">
-        <v>1.5</v>
-      </c>
-      <c r="D51">
-        <v>1.5</v>
-      </c>
-      <c r="E51">
-        <v>2</v>
-      </c>
-      <c r="F51">
-        <v>2</v>
-      </c>
-      <c r="G51">
-        <f t="shared" si="3"/>
-        <v>1.75</v>
-      </c>
-      <c r="I51">
-        <f t="shared" si="4"/>
-        <v>-1.75</v>
-      </c>
-      <c r="J51">
-        <f t="shared" si="5"/>
-        <v>-1.75</v>
-      </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>128</v>
-      </c>
-      <c r="B52" t="s">
-        <v>129</v>
-      </c>
-      <c r="C52">
-        <v>1</v>
-      </c>
-      <c r="D52">
-        <v>1</v>
-      </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-      <c r="F52">
-        <v>1</v>
-      </c>
-      <c r="G52">
-        <f t="shared" si="3"/>
-        <v>1</v>
-      </c>
-      <c r="I52">
-        <f t="shared" si="4"/>
-        <v>-1</v>
-      </c>
-      <c r="J52">
-        <f t="shared" si="5"/>
-        <v>-1</v>
-      </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A53" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B53" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C53">
-        <v>6</v>
-      </c>
-      <c r="D53">
-        <v>8</v>
-      </c>
-      <c r="E53">
-        <v>7</v>
-      </c>
-      <c r="F53">
-        <v>9</v>
-      </c>
-      <c r="G53">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>7.5</v>
-      </c>
-      <c r="I53">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-7.5</v>
-      </c>
-      <c r="J53">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-7.5</v>
-      </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A54" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B54" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C54" s="2">
-        <f>SUM(C55:C59)</f>
-        <v>47</v>
-      </c>
-      <c r="D54" s="2">
-        <f>SUM(D55:D59)</f>
-        <v>43</v>
-      </c>
-      <c r="E54" s="2">
-        <f>SUM(E55:E59)</f>
-        <v>44.5</v>
-      </c>
-      <c r="F54" s="2">
-        <f>SUM(F55:F59)</f>
-        <v>33.5</v>
-      </c>
-      <c r="G54" s="2">
-        <f>SUM(G55:G59)</f>
-        <v>42</v>
-      </c>
-      <c r="H54" s="2"/>
-      <c r="I54" s="2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-42</v>
-      </c>
-      <c r="J54" s="2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-42</v>
-      </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>62</v>
-      </c>
-      <c r="B55" t="s">
-        <v>87</v>
-      </c>
-      <c r="C55">
-        <v>4</v>
-      </c>
-      <c r="D55">
-        <v>4</v>
-      </c>
-      <c r="E55">
-        <v>7</v>
-      </c>
-      <c r="F55">
-        <v>5.5</v>
-      </c>
-      <c r="G55">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>5.125</v>
-      </c>
-      <c r="I55">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-5.125</v>
-      </c>
-      <c r="J55">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-5.125</v>
-      </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>63</v>
-      </c>
-      <c r="B56" t="s">
-        <v>86</v>
-      </c>
-      <c r="C56">
-        <v>6</v>
-      </c>
-      <c r="D56">
-        <v>8</v>
-      </c>
-      <c r="E56">
-        <v>6.5</v>
-      </c>
-      <c r="F56">
-        <v>5</v>
-      </c>
-      <c r="G56">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>6.375</v>
-      </c>
-      <c r="I56">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-6.375</v>
-      </c>
-      <c r="J56">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-6.375</v>
-      </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>64</v>
-      </c>
-      <c r="B57" t="s">
-        <v>85</v>
-      </c>
-      <c r="C57">
-        <v>2</v>
-      </c>
-      <c r="D57">
-        <v>1</v>
-      </c>
-      <c r="E57">
-        <v>1</v>
-      </c>
-      <c r="F57">
-        <v>1</v>
-      </c>
-      <c r="G57">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>1.25</v>
-      </c>
-      <c r="I57">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-1.25</v>
-      </c>
-      <c r="J57">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-1.25</v>
-      </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>65</v>
-      </c>
-      <c r="B58" t="s">
-        <v>91</v>
-      </c>
-      <c r="C58">
-        <v>25</v>
-      </c>
-      <c r="D58">
-        <v>20</v>
-      </c>
-      <c r="E58">
-        <v>20</v>
-      </c>
-      <c r="F58">
-        <v>15</v>
-      </c>
-      <c r="G58">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>20</v>
-      </c>
-      <c r="I58">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-20</v>
-      </c>
-      <c r="J58">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-20</v>
-      </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>81</v>
-      </c>
-      <c r="B59" t="s">
-        <v>80</v>
-      </c>
-      <c r="C59">
-        <v>10</v>
-      </c>
-      <c r="D59">
-        <v>10</v>
-      </c>
-      <c r="E59">
-        <v>10</v>
-      </c>
-      <c r="F59">
-        <v>7</v>
-      </c>
-      <c r="G59">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>9.25</v>
-      </c>
-      <c r="I59">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-9.25</v>
-      </c>
-      <c r="J59">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-9.25</v>
-      </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A60" s="2" t="s">
-        <v>66</v>
-      </c>
-      <c r="B60" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C60" s="2">
-        <f>SUM(C61:C62)</f>
-        <v>36</v>
-      </c>
-      <c r="D60" s="2">
-        <f>SUM(D61:D62)</f>
-        <v>28</v>
-      </c>
-      <c r="E60" s="2">
-        <f>SUM(E61:E62)</f>
-        <v>32</v>
-      </c>
-      <c r="F60" s="2">
-        <f>SUM(F61:F62)</f>
-        <v>25</v>
-      </c>
-      <c r="G60" s="2">
-        <f>SUM(G61:G62)</f>
-        <v>30.25</v>
-      </c>
-      <c r="H60" s="2"/>
-      <c r="I60" s="2">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-30.25</v>
-      </c>
-      <c r="J60" s="2">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-30.25</v>
-      </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>68</v>
-      </c>
-      <c r="B61" t="s">
-        <v>69</v>
-      </c>
-      <c r="C61">
-        <v>27</v>
-      </c>
-      <c r="D61">
-        <v>20</v>
-      </c>
-      <c r="E61">
-        <v>22</v>
-      </c>
-      <c r="F61">
-        <v>17</v>
-      </c>
-      <c r="G61">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>21.5</v>
-      </c>
-      <c r="I61">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
-        <v>-21.5</v>
-      </c>
-      <c r="J61">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-21.5</v>
-      </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>70</v>
-      </c>
-      <c r="B62" t="s">
-        <v>71</v>
-      </c>
-      <c r="C62">
-        <v>9</v>
-      </c>
-      <c r="D62">
-        <v>8</v>
-      </c>
-      <c r="E62">
-        <v>10</v>
-      </c>
-      <c r="F62">
-        <v>8</v>
-      </c>
-      <c r="G62">
-        <f>AVERAGE(Tabelle22[[#This Row],[Niklas]]:Tabelle22[[#This Row],[Eric]])</f>
-        <v>8.75</v>
-      </c>
-      <c r="I62">
-        <f>Tabelle22[[#This Row],[Ist-Stunden]]-Tabelle22[[#This Row],[Ø Schätzung (Soll-MA-Stunden)]]</f>
+        <f>Tabelle2[[#This Row],[Abweichung (Std.)]]</f>
         <v>-8.75</v>
       </c>
-      <c r="J62">
-        <f>Tabelle22[[#This Row],[Abweichung (Std.)]]</f>
-        <v>-8.75</v>
-      </c>
-    </row>
-    <row r="63" spans="1:10" ht="24" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A63" s="5"/>
-      <c r="B63" s="6" t="s">
+    </row>
+    <row r="49" spans="1:10" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A49" s="4"/>
+      <c r="B49" s="5" t="s">
         <v>97</v>
       </c>
-      <c r="C63" s="7">
-        <f>SUM(C60,C54,C25,C19,C15,C9,C2)</f>
+      <c r="C49" s="6">
+        <f>SUM(C46,C40,C25,C19,C15,C9,C2)</f>
         <v>416.5</v>
       </c>
-      <c r="D63" s="7">
-        <f>SUM(D60,D54,D25,D19,D15,D9,D2)</f>
+      <c r="D49" s="6">
+        <f>SUM(D46,D40,D25,D19,D15,D9,D2)</f>
         <v>465.5</v>
       </c>
-      <c r="E63" s="7">
-        <f>SUM(E60,E54,E25,E19,E15,E9,E2)</f>
+      <c r="E49" s="6">
+        <f>SUM(E46,E40,E25,E19,E15,E9,E2)</f>
         <v>404</v>
       </c>
-      <c r="F63" s="7">
-        <f>SUM(F60,F54,F25,F19,F15,F9,F2)</f>
+      <c r="F49" s="6">
+        <f>SUM(F46,F40,F25,F19,F15,F9,F2)</f>
         <v>429</v>
       </c>
-      <c r="G63" s="7">
-        <f>G60+G54+G25+G19+G15+G9+G2</f>
+      <c r="G49" s="6">
+        <f>G46+G40+G25+G19+G15+G9+G2</f>
         <v>428.75</v>
       </c>
-      <c r="H63" s="5"/>
-      <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
-    </row>
-    <row r="64" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+      <c r="H49" s="4"/>
+      <c r="I49" s="4"/>
+      <c r="J49" s="4"/>
+    </row>
+    <row r="50" spans="1:10" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.74803149606299213" right="0.74803149606299213" top="0.98425196850393704" bottom="0.98425196850393704" header="0.51181102362204722" footer="0.51181102362204722"/>
   <pageSetup paperSize="9" scale="61" fitToHeight="0" orientation="landscape" r:id="rId1"/>

</xml_diff>